<commit_message>
feat: implement file upload controllers and frontend views with database hash tracking and updated deployment configuration
</commit_message>
<xml_diff>
--- a/tests/MES.SPC.E2ETests/bin/Debug/net10.0/Fixtures/attribute_upload_valid.xlsx
+++ b/tests/MES.SPC.E2ETests/bin/Debug/net10.0/Fixtures/attribute_upload_valid.xlsx
@@ -64,22 +64,22 @@
     <x:t>DEF-001</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-05-21 03:26:59</x:t>
+    <x:t>2026-05-31 08:58:10</x:t>
   </x:si>
   <x:si>
     <x:t>E2E-OP-A</x:t>
   </x:si>
   <x:si>
-    <x:t>L-E2E-ATTR-20260521032659</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-05-21 03:16:59</x:t>
+    <x:t>L-E2E-ATTR-20260531085810</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-05-31 08:48:10</x:t>
   </x:si>
   <x:si>
     <x:t>E2E-OP-B</x:t>
   </x:si>
   <x:si>
-    <x:t>L-E2E-ATTR-20260521032659-2</x:t>
+    <x:t>L-E2E-ATTR-20260531085810-2</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
feat: implement SPC rule engine tests and add E2E utility fixtures for excel data integration
</commit_message>
<xml_diff>
--- a/tests/MES.SPC.E2ETests/bin/Debug/net10.0/Fixtures/attribute_upload_valid.xlsx
+++ b/tests/MES.SPC.E2ETests/bin/Debug/net10.0/Fixtures/attribute_upload_valid.xlsx
@@ -64,22 +64,22 @@
     <x:t>DEF-001</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-05-31 08:58:10</x:t>
+    <x:t>2026-06-08 09:11:38</x:t>
   </x:si>
   <x:si>
     <x:t>E2E-OP-A</x:t>
   </x:si>
   <x:si>
-    <x:t>L-E2E-ATTR-20260531085810</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-05-31 08:48:10</x:t>
+    <x:t>L-E2E-ATTR-20260608091138</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-06-08 09:01:38</x:t>
   </x:si>
   <x:si>
     <x:t>E2E-OP-B</x:t>
   </x:si>
   <x:si>
-    <x:t>L-E2E-ATTR-20260531085810-2</x:t>
+    <x:t>L-E2E-ATTR-20260608091138-2</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>